<commit_message>
Clarify DMS-04 and Dispute Triage ownership per feedback
DMS-04 previously implied the system determines fraud/non-fraud
classification and routes automatically; the classification is actually
an agent/process decision made during intake. Revised to describe the
system's actual responsibility: capturing the agent's classification and
queuing the case to the corresponding team accordingly.

Updated the Dispute Triage stage header to note it's executed by whichever
team (Fraud or Payment Services) was assigned at intake, rather than a
separate unified triage function.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Beem Visa Debit - Dispute Management System Requirements.xlsx
+++ b/Beem Visa Debit - Dispute Management System Requirements.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>The Dispute Management System shall route a case to the Fraud team or the Payment Services team automatically, based on the agent's response to whether the member recognizes the transaction.</t>
+          <t>The Dispute Management System shall capture the agent's fraud/non-fraud classification of the dispute and queue the case to the corresponding team (Fraud or Payment Services) based on the recorded classification.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -657,7 +657,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2. Dispute Triage</t>
+          <t>2. Dispute Triage (executed by the team assigned at intake: Fraud or Payment Services)</t>
         </is>
       </c>
       <c r="B13" s="5" t="n"/>

</xml_diff>